<commit_message>
fixed missing lioness season in title
</commit_message>
<xml_diff>
--- a/content/database.xlsx
+++ b/content/database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hannah\life\dabad2_0\dabad\content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C6A8CD00-7839-4EEE-85EA-7B142AA417E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B13AF9A-0EB4-445D-8DE2-A65563CF2937}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{730DD696-8E95-48A8-8025-F5D06081233D}"/>
   </bookViews>
@@ -8722,9 +8722,6 @@
     <t>Lioness_Season_2_2024</t>
   </si>
   <si>
-    <t>Lioness</t>
-  </si>
-  <si>
     <t>Lioness [Season 1], Lioness [Season 3]</t>
   </si>
   <si>
@@ -8744,6 +8741,9 @@
   </si>
   <si>
     <t>Jurassic World: Rebirth</t>
+  </si>
+  <si>
+    <t>Lioness [Season 2]</t>
   </si>
 </sst>
 </file>
@@ -9227,7 +9227,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -9270,7 +9270,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -13578,7 +13577,7 @@
         <v>26</v>
       </c>
       <c r="M79" s="4" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N79" s="6">
         <v>148</v>
@@ -13631,7 +13630,7 @@
         <v>26</v>
       </c>
       <c r="M80" s="4" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N80" s="6">
         <v>124</v>
@@ -18486,7 +18485,7 @@
         <v>26</v>
       </c>
       <c r="M177" s="4" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N177" s="6">
         <v>129</v>
@@ -19847,7 +19846,7 @@
         <v>26</v>
       </c>
       <c r="M204" s="4" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N204" s="6">
         <v>96</v>
@@ -20567,7 +20566,7 @@
         <v>26</v>
       </c>
       <c r="M218" s="4" t="s">
-        <v>2905</v>
+        <v>2904</v>
       </c>
       <c r="N218" s="6">
         <v>78</v>
@@ -20618,7 +20617,7 @@
         <v>26</v>
       </c>
       <c r="M219" s="4" t="s">
-        <v>2905</v>
+        <v>2904</v>
       </c>
       <c r="N219" s="6">
         <v>89</v>
@@ -22156,7 +22155,7 @@
         <v>26</v>
       </c>
       <c r="M251" s="4" t="s">
-        <v>2905</v>
+        <v>2904</v>
       </c>
       <c r="N251" s="6">
         <v>98</v>
@@ -31090,7 +31089,7 @@
         <v>26</v>
       </c>
       <c r="M431" s="4" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N431" s="6">
         <v>127</v>
@@ -31143,7 +31142,7 @@
         <v>26</v>
       </c>
       <c r="M432" s="4" t="s">
-        <v>2906</v>
+        <v>2905</v>
       </c>
       <c r="N432" s="6">
         <v>129</v>
@@ -34295,7 +34294,7 @@
         <v>29</v>
       </c>
       <c r="D496" s="14" t="s">
-        <v>2899</v>
+        <v>2906</v>
       </c>
       <c r="E496" s="7">
         <v>2024</v>
@@ -34312,8 +34311,8 @@
       <c r="L496" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="M496" s="16" t="s">
-        <v>2900</v>
+      <c r="M496" t="s">
+        <v>2899</v>
       </c>
       <c r="N496" s="7">
         <v>42</v>
@@ -34325,16 +34324,16 @@
         <v>2257</v>
       </c>
       <c r="R496" s="2" t="s">
+        <v>2901</v>
+      </c>
+      <c r="S496" t="s">
+        <v>2900</v>
+      </c>
+      <c r="T496" t="s">
         <v>2902</v>
       </c>
-      <c r="S496" t="s">
-        <v>2901</v>
-      </c>
-      <c r="T496" t="s">
+      <c r="U496" t="s">
         <v>2903</v>
-      </c>
-      <c r="U496" t="s">
-        <v>2904</v>
       </c>
     </row>
     <row r="497" spans="1:21" x14ac:dyDescent="0.3">

</xml_diff>